<commit_message>
config and small bug fix
</commit_message>
<xml_diff>
--- a/input/EUROMODpolicySchedule.xlsx
+++ b/input/EUROMODpolicySchedule.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10503"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <mc:AlternateContent>
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Sonnewald/GitHub/SimPaths/input/"/>
     </mc:Choice>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="24">
   <si>
     <t>Filename</t>
   </si>
@@ -52,12 +52,58 @@
   </si>
   <si>
     <t>2030</t>
+  </si>
+  <si>
+    <t>uk_2011_std.txt</t>
+  </si>
+  <si>
+    <t>uk_2012_std.txt</t>
+  </si>
+  <si>
+    <t>uk_2013_std.txt</t>
+  </si>
+  <si>
+    <t>uk_2014_std.txt</t>
+  </si>
+  <si>
+    <t>uk_2016_std.txt</t>
+  </si>
+  <si>
+    <t>uk_2017_std.txt</t>
+  </si>
+  <si>
+    <t>uk_2018_std.txt</t>
+  </si>
+  <si>
+    <t>uk_2019_std.txt</t>
+  </si>
+  <si>
+    <t>uk_2020_std.txt</t>
+  </si>
+  <si>
+    <t>uk_2021_std.txt</t>
+  </si>
+  <si>
+    <t>uk_2022_std.txt</t>
+  </si>
+  <si>
+    <t>uk_2023_std.txt</t>
+  </si>
+  <si>
+    <t>uk_2024_std.txt</t>
+  </si>
+  <si>
+    <t>uk_2025_std.txt</t>
+  </si>
+  <si>
+    <t>uk_2026_std.txt</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="0"/>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -403,14 +449,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C5CC6207-DD24-427A-A7C5-E1B68985A6D0}">
-  <dimension ref="A1:AMK3"/>
+  <dimension ref="A1:D18"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="17.83203125" customWidth="1" collapsed="1"/>
-    <col min="2" max="1025" width="9.1640625" collapsed="1"/>
+    <col min="1" max="1" customWidth="true" width="17.83203125" collapsed="true"/>
+    <col min="2" max="1025" width="9.1640625" collapsed="true"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -424,31 +470,241 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="2">
       <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C3" t="s">
+        <v>4</v>
+      </c>
+      <c r="D3" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D4" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" t="s">
+        <v>4</v>
+      </c>
+      <c r="C5" t="s">
+        <v>4</v>
+      </c>
+      <c r="D5" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
         <v>5</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B6" t="s">
         <v>3</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C6" t="s">
         <v>3</v>
       </c>
-      <c r="D2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
+      <c r="D6" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" t="s">
+        <v>4</v>
+      </c>
+      <c r="C7" t="s">
+        <v>4</v>
+      </c>
+      <c r="D7" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B8" t="s">
+        <v>4</v>
+      </c>
+      <c r="C8" t="s">
+        <v>4</v>
+      </c>
+      <c r="D8" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>15</v>
+      </c>
+      <c r="B9" t="s">
+        <v>4</v>
+      </c>
+      <c r="C9" t="s">
+        <v>4</v>
+      </c>
+      <c r="D9" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>16</v>
+      </c>
+      <c r="B10" t="s">
+        <v>4</v>
+      </c>
+      <c r="C10" t="s">
+        <v>4</v>
+      </c>
+      <c r="D10" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>17</v>
+      </c>
+      <c r="B11" t="s">
+        <v>4</v>
+      </c>
+      <c r="C11" t="s">
+        <v>4</v>
+      </c>
+      <c r="D11" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s">
+        <v>18</v>
+      </c>
+      <c r="B12" t="s">
+        <v>4</v>
+      </c>
+      <c r="C12" t="s">
+        <v>4</v>
+      </c>
+      <c r="D12" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s">
+        <v>19</v>
+      </c>
+      <c r="B13" t="s">
+        <v>4</v>
+      </c>
+      <c r="C13" t="s">
+        <v>4</v>
+      </c>
+      <c r="D13" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s">
+        <v>20</v>
+      </c>
+      <c r="B14" t="s">
+        <v>4</v>
+      </c>
+      <c r="C14" t="s">
+        <v>4</v>
+      </c>
+      <c r="D14" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s">
+        <v>21</v>
+      </c>
+      <c r="B15" t="s">
+        <v>4</v>
+      </c>
+      <c r="C15" t="s">
+        <v>4</v>
+      </c>
+      <c r="D15" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s">
+        <v>22</v>
+      </c>
+      <c r="B16" t="s">
+        <v>4</v>
+      </c>
+      <c r="C16" t="s">
+        <v>4</v>
+      </c>
+      <c r="D16" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s">
+        <v>23</v>
+      </c>
+      <c r="B17" t="s">
+        <v>4</v>
+      </c>
+      <c r="C17" t="s">
+        <v>4</v>
+      </c>
+      <c r="D17" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s">
         <v>7</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B18" t="s">
         <v>8</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C18" t="s">
         <v>8</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D18" t="s">
         <v>4</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Revert "config and small bug fix"
This reverts commit f0e8891c537aadde3e02a4dc39ab63d0e7ee4186.
</commit_message>
<xml_diff>
--- a/input/EUROMODpolicySchedule.xlsx
+++ b/input/EUROMODpolicySchedule.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10503"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Sonnewald/GitHub/SimPaths/input/"/>
     </mc:Choice>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="9">
   <si>
     <t>Filename</t>
   </si>
@@ -52,58 +52,12 @@
   </si>
   <si>
     <t>2030</t>
-  </si>
-  <si>
-    <t>uk_2011_std.txt</t>
-  </si>
-  <si>
-    <t>uk_2012_std.txt</t>
-  </si>
-  <si>
-    <t>uk_2013_std.txt</t>
-  </si>
-  <si>
-    <t>uk_2014_std.txt</t>
-  </si>
-  <si>
-    <t>uk_2016_std.txt</t>
-  </si>
-  <si>
-    <t>uk_2017_std.txt</t>
-  </si>
-  <si>
-    <t>uk_2018_std.txt</t>
-  </si>
-  <si>
-    <t>uk_2019_std.txt</t>
-  </si>
-  <si>
-    <t>uk_2020_std.txt</t>
-  </si>
-  <si>
-    <t>uk_2021_std.txt</t>
-  </si>
-  <si>
-    <t>uk_2022_std.txt</t>
-  </si>
-  <si>
-    <t>uk_2023_std.txt</t>
-  </si>
-  <si>
-    <t>uk_2024_std.txt</t>
-  </si>
-  <si>
-    <t>uk_2025_std.txt</t>
-  </si>
-  <si>
-    <t>uk_2026_std.txt</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="0"/>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -449,14 +403,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C5CC6207-DD24-427A-A7C5-E1B68985A6D0}">
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:AMK3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="17.83203125" collapsed="true"/>
-    <col min="2" max="1025" width="9.1640625" collapsed="true"/>
+    <col min="1" max="1" width="17.83203125" customWidth="1" collapsed="1"/>
+    <col min="2" max="1025" width="9.1640625" collapsed="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -470,241 +424,31 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="B2" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C2" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="B3" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="C3" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="D3" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="s">
-        <v>11</v>
-      </c>
-      <c r="B4" t="s">
-        <v>4</v>
-      </c>
-      <c r="C4" t="s">
-        <v>4</v>
-      </c>
-      <c r="D4" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="s">
-        <v>12</v>
-      </c>
-      <c r="B5" t="s">
-        <v>4</v>
-      </c>
-      <c r="C5" t="s">
-        <v>4</v>
-      </c>
-      <c r="D5" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="s">
-        <v>5</v>
-      </c>
-      <c r="B6" t="s">
-        <v>3</v>
-      </c>
-      <c r="C6" t="s">
-        <v>3</v>
-      </c>
-      <c r="D6" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="s">
-        <v>13</v>
-      </c>
-      <c r="B7" t="s">
-        <v>4</v>
-      </c>
-      <c r="C7" t="s">
-        <v>4</v>
-      </c>
-      <c r="D7" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="s">
-        <v>14</v>
-      </c>
-      <c r="B8" t="s">
-        <v>4</v>
-      </c>
-      <c r="C8" t="s">
-        <v>4</v>
-      </c>
-      <c r="D8" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="s">
-        <v>15</v>
-      </c>
-      <c r="B9" t="s">
-        <v>4</v>
-      </c>
-      <c r="C9" t="s">
-        <v>4</v>
-      </c>
-      <c r="D9" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="s">
-        <v>16</v>
-      </c>
-      <c r="B10" t="s">
-        <v>4</v>
-      </c>
-      <c r="C10" t="s">
-        <v>4</v>
-      </c>
-      <c r="D10" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="s">
-        <v>17</v>
-      </c>
-      <c r="B11" t="s">
-        <v>4</v>
-      </c>
-      <c r="C11" t="s">
-        <v>4</v>
-      </c>
-      <c r="D11" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="s">
-        <v>18</v>
-      </c>
-      <c r="B12" t="s">
-        <v>4</v>
-      </c>
-      <c r="C12" t="s">
-        <v>4</v>
-      </c>
-      <c r="D12" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="s">
-        <v>19</v>
-      </c>
-      <c r="B13" t="s">
-        <v>4</v>
-      </c>
-      <c r="C13" t="s">
-        <v>4</v>
-      </c>
-      <c r="D13" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="s">
-        <v>20</v>
-      </c>
-      <c r="B14" t="s">
-        <v>4</v>
-      </c>
-      <c r="C14" t="s">
-        <v>4</v>
-      </c>
-      <c r="D14" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="s">
-        <v>21</v>
-      </c>
-      <c r="B15" t="s">
-        <v>4</v>
-      </c>
-      <c r="C15" t="s">
-        <v>4</v>
-      </c>
-      <c r="D15" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="s">
-        <v>22</v>
-      </c>
-      <c r="B16" t="s">
-        <v>4</v>
-      </c>
-      <c r="C16" t="s">
-        <v>4</v>
-      </c>
-      <c r="D16" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="s">
-        <v>23</v>
-      </c>
-      <c r="B17" t="s">
-        <v>4</v>
-      </c>
-      <c r="C17" t="s">
-        <v>4</v>
-      </c>
-      <c r="D17" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="s">
-        <v>7</v>
-      </c>
-      <c r="B18" t="s">
-        <v>8</v>
-      </c>
-      <c r="C18" t="s">
-        <v>8</v>
-      </c>
-      <c r="D18" t="s">
         <v>4</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Reapply "config and small bug fix"
This reverts commit a7051b1e1ce98d1a648a331694b5434626113b6f.
</commit_message>
<xml_diff>
--- a/input/EUROMODpolicySchedule.xlsx
+++ b/input/EUROMODpolicySchedule.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10503"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <mc:AlternateContent>
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Sonnewald/GitHub/SimPaths/input/"/>
     </mc:Choice>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="24">
   <si>
     <t>Filename</t>
   </si>
@@ -52,12 +52,58 @@
   </si>
   <si>
     <t>2030</t>
+  </si>
+  <si>
+    <t>uk_2011_std.txt</t>
+  </si>
+  <si>
+    <t>uk_2012_std.txt</t>
+  </si>
+  <si>
+    <t>uk_2013_std.txt</t>
+  </si>
+  <si>
+    <t>uk_2014_std.txt</t>
+  </si>
+  <si>
+    <t>uk_2016_std.txt</t>
+  </si>
+  <si>
+    <t>uk_2017_std.txt</t>
+  </si>
+  <si>
+    <t>uk_2018_std.txt</t>
+  </si>
+  <si>
+    <t>uk_2019_std.txt</t>
+  </si>
+  <si>
+    <t>uk_2020_std.txt</t>
+  </si>
+  <si>
+    <t>uk_2021_std.txt</t>
+  </si>
+  <si>
+    <t>uk_2022_std.txt</t>
+  </si>
+  <si>
+    <t>uk_2023_std.txt</t>
+  </si>
+  <si>
+    <t>uk_2024_std.txt</t>
+  </si>
+  <si>
+    <t>uk_2025_std.txt</t>
+  </si>
+  <si>
+    <t>uk_2026_std.txt</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="0"/>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -403,14 +449,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C5CC6207-DD24-427A-A7C5-E1B68985A6D0}">
-  <dimension ref="A1:AMK3"/>
+  <dimension ref="A1:D18"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="17.83203125" customWidth="1" collapsed="1"/>
-    <col min="2" max="1025" width="9.1640625" collapsed="1"/>
+    <col min="1" max="1" customWidth="true" width="17.83203125" collapsed="true"/>
+    <col min="2" max="1025" width="9.1640625" collapsed="true"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -424,31 +470,241 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="2">
       <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C3" t="s">
+        <v>4</v>
+      </c>
+      <c r="D3" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D4" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" t="s">
+        <v>4</v>
+      </c>
+      <c r="C5" t="s">
+        <v>4</v>
+      </c>
+      <c r="D5" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
         <v>5</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B6" t="s">
         <v>3</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C6" t="s">
         <v>3</v>
       </c>
-      <c r="D2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
+      <c r="D6" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" t="s">
+        <v>4</v>
+      </c>
+      <c r="C7" t="s">
+        <v>4</v>
+      </c>
+      <c r="D7" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B8" t="s">
+        <v>4</v>
+      </c>
+      <c r="C8" t="s">
+        <v>4</v>
+      </c>
+      <c r="D8" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>15</v>
+      </c>
+      <c r="B9" t="s">
+        <v>4</v>
+      </c>
+      <c r="C9" t="s">
+        <v>4</v>
+      </c>
+      <c r="D9" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>16</v>
+      </c>
+      <c r="B10" t="s">
+        <v>4</v>
+      </c>
+      <c r="C10" t="s">
+        <v>4</v>
+      </c>
+      <c r="D10" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>17</v>
+      </c>
+      <c r="B11" t="s">
+        <v>4</v>
+      </c>
+      <c r="C11" t="s">
+        <v>4</v>
+      </c>
+      <c r="D11" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s">
+        <v>18</v>
+      </c>
+      <c r="B12" t="s">
+        <v>4</v>
+      </c>
+      <c r="C12" t="s">
+        <v>4</v>
+      </c>
+      <c r="D12" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s">
+        <v>19</v>
+      </c>
+      <c r="B13" t="s">
+        <v>4</v>
+      </c>
+      <c r="C13" t="s">
+        <v>4</v>
+      </c>
+      <c r="D13" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s">
+        <v>20</v>
+      </c>
+      <c r="B14" t="s">
+        <v>4</v>
+      </c>
+      <c r="C14" t="s">
+        <v>4</v>
+      </c>
+      <c r="D14" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s">
+        <v>21</v>
+      </c>
+      <c r="B15" t="s">
+        <v>4</v>
+      </c>
+      <c r="C15" t="s">
+        <v>4</v>
+      </c>
+      <c r="D15" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s">
+        <v>22</v>
+      </c>
+      <c r="B16" t="s">
+        <v>4</v>
+      </c>
+      <c r="C16" t="s">
+        <v>4</v>
+      </c>
+      <c r="D16" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s">
+        <v>23</v>
+      </c>
+      <c r="B17" t="s">
+        <v>4</v>
+      </c>
+      <c r="C17" t="s">
+        <v>4</v>
+      </c>
+      <c r="D17" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s">
         <v>7</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B18" t="s">
         <v>8</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C18" t="s">
         <v>8</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D18" t="s">
         <v>4</v>
       </c>
     </row>

</xml_diff>